<commit_message>
site build 2026-10-09 07:30
</commit_message>
<xml_diff>
--- a/models/sovereigns/Qatar_Sovereign_Model.xlsx
+++ b/models/sovereigns/Qatar_Sovereign_Model.xlsx
@@ -647,12 +647,12 @@
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>IMF MFS interest rates</t>
+          <t>IMF MFS</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
@@ -660,11 +660,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
-        <is>
-          <t>IMF MFS interest rates, monetary policy-related rate, % p.a., monthly (auto-filled; a run's sourced point replaces it unless older)</t>
-        </is>
-      </c>
+      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -690,7 +686,7 @@
         </is>
       </c>
       <c r="B5" s="2" t="n">
-        <v>0.7338</v>
+        <v>0.73</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -699,7 +695,7 @@
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>2025-08</t>
+          <t>Aug-25</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -712,11 +708,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr">
-        <is>
-          <t>IMF CPI database, all items, y/y % change, monthly (auto-filled; a run's sourced point replaces it unless older)</t>
-        </is>
-      </c>
+      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -739,7 +731,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (repo data)</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
@@ -747,11 +739,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -791,7 +779,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (repo data)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
@@ -801,7 +789,7 @@
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
+          <t>IMF WEO general government debt</t>
         </is>
       </c>
     </row>
@@ -843,7 +831,7 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (repo data)</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
@@ -851,11 +839,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -929,7 +913,7 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (repo data)</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
@@ -937,11 +921,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -985,7 +965,7 @@
         </is>
       </c>
       <c r="B16" s="2" t="n">
-        <v>61.098</v>
+        <v>61.1</v>
       </c>
       <c r="C16" t="inlineStr">
         <is>
@@ -994,7 +974,7 @@
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>2026-08</t>
+          <t>Aug-26</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
@@ -1009,7 +989,7 @@
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Gross official reserves incl. gold at national valuation, end-month (auto-filled; a run's sourced point replaces it unless older)</t>
+          <t>gross incl. gold (FX ex gold 44.6, gold 16.5)</t>
         </is>
       </c>
     </row>
@@ -1037,7 +1017,7 @@
         </is>
       </c>
       <c r="B18" s="2" t="n">
-        <v>7.453</v>
+        <v>7.45</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -1059,11 +1039,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1123,7 +1099,7 @@
         </is>
       </c>
       <c r="B22" s="2" t="n">
-        <v>217.416</v>
+        <v>217.4</v>
       </c>
       <c r="C22" t="inlineStr">
         <is>
@@ -1137,7 +1113,7 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>IMF WEO</t>
+          <t>IMF WEO (repo data)</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
@@ -1145,11 +1121,7 @@
           <t>09-Oct-26</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr">
-        <is>
-          <t>official annual series (filled automatically; a run's sourced point replaces it)</t>
-        </is>
-      </c>
+      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1245,6 +1217,21 @@
       <c r="A29" t="inlineStr">
         <is>
           <t>fitch</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>AA</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>Negative</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>06-May-26</t>
         </is>
       </c>
     </row>
@@ -1280,7 +1267,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B12"/>
+  <dimension ref="A1:C12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -1294,6 +1281,11 @@
       </c>
       <c r="B1" s="1" t="inlineStr">
         <is>
+          <t>2026E</t>
+        </is>
+      </c>
+      <c r="C1" s="1" t="inlineStr">
+        <is>
           <t>Source</t>
         </is>
       </c>
@@ -1304,7 +1296,14 @@
           <t>nominal_gdp_usd_bn</t>
         </is>
       </c>
-      <c r="B2" t="inlineStr"/>
+      <c r="B2" s="2" t="n">
+        <v>217.4</v>
+      </c>
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>IMF WEO (repo data), 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1312,7 +1311,14 @@
           <t>real_gdp_growth_pct</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr"/>
+      <c r="B3" s="2" t="n">
+        <v>-8.6</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>IMF WEO (repo data), 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1320,7 +1326,8 @@
           <t>cpi_avg_pct</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" s="2" t="n"/>
+      <c r="C4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -1328,7 +1335,14 @@
           <t>current_account_pct_gdp</t>
         </is>
       </c>
-      <c r="B5" t="inlineStr"/>
+      <c r="B5" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>IMF WEO (repo data), 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -1336,7 +1350,14 @@
           <t>fiscal_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B6" t="inlineStr"/>
+      <c r="B6" s="2" t="n">
+        <v>-3.4</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>IMF WEO (repo data), 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -1344,7 +1365,8 @@
           <t>primary_balance_pct_gdp</t>
         </is>
       </c>
-      <c r="B7" t="inlineStr"/>
+      <c r="B7" s="2" t="n"/>
+      <c r="C7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -1352,7 +1374,14 @@
           <t>gov_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B8" t="inlineStr"/>
+      <c r="B8" s="2" t="n">
+        <v>43.3</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>IMF WEO (repo data), 09-Oct-26</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -1360,7 +1389,8 @@
           <t>external_debt_pct_gdp</t>
         </is>
       </c>
-      <c r="B9" t="inlineStr"/>
+      <c r="B9" s="2" t="n"/>
+      <c r="C9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -1368,7 +1398,8 @@
           <t>gross_reserves_usd_bn</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr"/>
+      <c r="B10" s="2" t="n"/>
+      <c r="C10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -1376,7 +1407,8 @@
           <t>revenue_pct_gdp</t>
         </is>
       </c>
-      <c r="B11" t="inlineStr"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -1384,7 +1416,8 @@
           <t>interest_pct_revenue</t>
         </is>
       </c>
-      <c r="B12" t="inlineStr"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>